<commit_message>
Verify: delete all outputs, re-run from scratch, confirm match
Deleted all outputs/ files, re-ran every script end-to-end:
- 01_adoption_model.py through consolidate_outputs.py (Task 1)
- 02_top_down_funnel.py (Task 2 — 17/17 sanity checks PASS)
- 15/15 pytest tests pass
- PDF rebuilt

All regenerated values match the case study document exactly.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/task1_adoption/task1_outputs.xlsx
+++ b/outputs/task1_adoption/task1_outputs.xlsx
@@ -988,7 +988,7 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>Active beta-blocker
-(within 90 days)</t>
+(30-day coverage window)</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1013,7 +1013,7 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>Active CCB prescription
-(within 90 days)</t>
+(30-day coverage window)</t>
         </is>
       </c>
       <c r="C5" t="n">

</xml_diff>